<commit_message>
Ajustes: citas con audio, ratas en fauna, próximos pasos con validaciones, ficha en lenguaje sencillo, inicio desde la lámina 1
</commit_message>
<xml_diff>
--- a/RECOEVO_Estudio_Campo/03_Base_de_Datos/RECOEVO_Base_de_Datos_Campo.xlsx
+++ b/RECOEVO_Estudio_Campo/03_Base_de_Datos/RECOEVO_Base_de_Datos_Campo.xlsx
@@ -292,14 +292,13 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Participantes" displayName="Participantes" ref="A1:E9" headerRowCount="1">
-  <autoFilter ref="A1:E9"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Participantes" displayName="Participantes" ref="A1:D9" headerRowCount="1">
+  <autoFilter ref="A1:D9"/>
+  <tableColumns count="4">
     <tableColumn id="1" name="Código"/>
     <tableColumn id="2" name="Rol"/>
     <tableColumn id="3" name="Perfil (anonimizado)"/>
     <tableColumn id="4" name="Grabaciones"/>
-    <tableColumn id="5" name="Género"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
@@ -630,7 +629,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>5 hombres, 3 mujeres · 3 hogares, 3 comercios, 2 mixtos</t>
+          <t>3 hogares, 3 comercios, 2 hogar y comercio</t>
         </is>
       </c>
     </row>
@@ -830,14 +829,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -861,11 +859,6 @@
           <t>Grabaciones</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Género</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -888,11 +881,6 @@
           <t>Audio1</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -915,11 +903,6 @@
           <t>Audio2 + Audio3</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -942,11 +925,6 @@
           <t>Audio4</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -969,11 +947,6 @@
           <t>Audio5</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -996,11 +969,6 @@
           <t>Audio6 + Audio10</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1015,17 +983,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Residente adulta mayor, vive con su hija</t>
+          <t>Residente adulto mayor, vive con su hija</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Audio7</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>M</t>
         </is>
       </c>
     </row>
@@ -1050,11 +1013,6 @@
           <t>Audio8</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1075,11 +1033,6 @@
       <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Audio9</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>H</t>
         </is>
       </c>
     </row>

</xml_diff>